<commit_message>
Adapta el kit a la flota real: LGV, satélites, conveyors, Joloda y cargadores
Reemplaza el catálogo de ejemplo por los 20 equipos reales del CD: 5 LGV,
7 satélites, 2 conveyors, 1 Joloda, 2 racks de cargadores de satélites y
3 cargadores de LGV. Reescribe bitácora, fallas y plan mensual de ejemplo
con actividades propias de esa flota (navegación LGV, rescate de satélites,
baterías y carga, hidráulica del Joloda), agrega los tipos de falla
Hidráulica y Batería/Carga, la actividad Cambio de Batería, y actualiza
las maquetas de las 3 páginas del dashboard.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VZDcZPRf2zrYzCo4cb6M6C
</commit_message>
<xml_diff>
--- a/powerbi-mantencion/plantilla/Plantilla_Bitacora_Mantencion.xlsx
+++ b/powerbi-mantencion/plantilla/Plantilla_Bitacora_Mantencion.xlsx
@@ -737,7 +737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -984,7 +984,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Neumática</t>
+          <t>Hidráulica</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -1011,7 +1011,7 @@
     <row r="6">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Reparación</t>
+          <t>Cambio de Batería</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -1033,12 +1033,12 @@
     <row r="7">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Mantención Preventiva</t>
+          <t>Reparación</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Operacional</t>
+          <t>Batería / Carga</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
@@ -1050,19 +1050,31 @@
     <row r="8">
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Apoyo a Operación</t>
+          <t>Mantención Preventiva</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Operacional</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Capacitación</t>
+          <t>Apoyo a Operación</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Capacitación</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Otro</t>
         </is>
@@ -1079,7 +1091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1131,22 +1143,22 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-01</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Sorter principal cross-belt</t>
+          <t>LGV 01</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Clasificador</t>
+          <t>LGV</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>Clasificación</t>
+          <t>Circuito LGV</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -1156,7 +1168,7 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>Vanderlande</t>
+          <t>Elettric80</t>
         </is>
       </c>
       <c r="G2" s="7" t="n">
@@ -1166,32 +1178,32 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>TRK-01</t>
+          <t>LGV-02</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Transportador recepción L1</t>
+          <t>LGV 02</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Transportador</t>
+          <t>LGV</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Recepción</t>
+          <t>Circuito LGV</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Interroll</t>
+          <t>Elettric80</t>
         </is>
       </c>
       <c r="G3" s="7" t="n">
@@ -1201,22 +1213,22 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>TRK-02</t>
+          <t>LGV-03</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Transportador salida muelles</t>
+          <t>LGV 03</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Transportador</t>
+          <t>LGV</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Despacho</t>
+          <t>Circuito LGV</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -1226,7 +1238,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Interroll</t>
+          <t>Elettric80</t>
         </is>
       </c>
       <c r="G4" s="7" t="n">
@@ -1236,22 +1248,22 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>TRK-03</t>
+          <t>LGV-04</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Transportador espina central</t>
+          <t>LGV 04</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Transportador</t>
+          <t>LGV</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Clasificación</t>
+          <t>Circuito LGV</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -1261,7 +1273,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>BEUMER</t>
+          <t>Elettric80</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -1271,22 +1283,22 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>PAL-01</t>
+          <t>LGV-05</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Paletizador robótico 1</t>
+          <t>LGV 05</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Robot paletizado</t>
+          <t>LGV</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Despacho</t>
+          <t>Circuito LGV</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -1296,7 +1308,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>KUKA</t>
+          <t>Elettric80</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -1306,22 +1318,22 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>PAL-02</t>
+          <t>SAT-01</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Paletizador robótico 2</t>
+          <t>Satélite 01</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Robot paletizado</t>
+          <t>Satélite</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Despacho</t>
+          <t>Bodega de racks</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1331,102 +1343,102 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>KUKA</t>
+          <t>Automha</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>TRE-01</t>
+          <t>SAT-02</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Transelevador pasillo A</t>
+          <t>Satélite 02</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>ASRS</t>
+          <t>Satélite</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Bodega automática</t>
+          <t>Bodega de racks</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Mecalux</t>
+          <t>Automha</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>TRE-02</t>
+          <t>SAT-03</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Transelevador pasillo B</t>
+          <t>Satélite 03</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>ASRS</t>
+          <t>Satélite</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Bodega automática</t>
+          <t>Bodega de racks</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Mecalux</t>
+          <t>Automha</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>SAT-04</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Enfardadora automática</t>
+          <t>Satélite 04</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Enfardadora</t>
+          <t>Satélite</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Despacho</t>
+          <t>Bodega de racks</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -1436,32 +1448,32 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Robopac</t>
+          <t>Automha</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>2019</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>ETI-01</t>
+          <t>SAT-05</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Etiquetadora print &amp; apply</t>
+          <t>Satélite 05</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Etiquetadora</t>
+          <t>Satélite</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Clasificación</t>
+          <t>Bodega de racks</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1471,32 +1483,32 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Videojet</t>
+          <t>Automha</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>ELE-01</t>
+          <t>SAT-06</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Elevador de cajas mezanina</t>
+          <t>Satélite 06</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Elevador</t>
+          <t>Satélite</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Bodega automática</t>
+          <t>Bodega de racks</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -1506,46 +1518,326 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Qimarox</t>
+          <t>Automha</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>BSC-01</t>
+          <t>SAT-07</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Checkweigher línea salida</t>
+          <t>Satélite 07</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Báscula dinámica</t>
+          <t>Satélite</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Despacho</t>
+          <t>Bodega de racks</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Mettler Toledo</t>
+          <t>Automha</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
-        <v>2023</v>
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>CNV-01</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Conveyor entrada producción</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Conveyor</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Recepción producción</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Interroll</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>CNV-02</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Conveyor salida a andenes</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Conveyor</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Despacho / Andenes</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Interroll</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>JOL-01</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Joloda carga automática de camiones</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Joloda</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Despacho / Andenes</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Joloda Hydraroll</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>RCS-01</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Rack cargadores de satélites 1</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Cargador satélites</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Sala de carga</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Fronius</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>RCS-02</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Rack cargadores de satélites 2</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Cargador satélites</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Sala de carga</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Fronius</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>CLG-01</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Cargador LGV 1</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Cargador LGV</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Sala de carga</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>Elettric80</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>CLG-02</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Cargador LGV 2</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Cargador LGV</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Sala de carga</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Elettric80</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>CLG-03</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Cargador LGV 3</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Cargador LGV</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Sala de carga</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Elettric80</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="n">
+        <v>2022</v>
       </c>
     </row>
   </sheetData>
@@ -1648,7 +1940,7 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-01</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -1658,7 +1950,7 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>Ronda de inicio de turno: revisión de carros y bandas del sorter, sin novedades.</t>
+          <t>Ronda de inicio de turno: circuito LGV, cruces y reflectores sin novedades.</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
@@ -1692,7 +1984,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>TRK-01</t>
+          <t>CNV-01</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -1702,7 +1994,7 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Limpieza de fotoceldas y retiro de film atrapado en curva C2.</t>
+          <t>Limpieza de fotoceldas y retiro de film atrapado en transferencia T2.</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -1736,7 +2028,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>PAL-01</t>
+          <t>SAT-03</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -1746,7 +2038,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Ajuste de garra: presión de vacío baja en ventosas, se regula a 0,6 bar.</t>
+          <t>Ajuste de topes de entrada en calle 12: el satélite entraba desalineado.</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1764,7 +2056,7 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>Vigilar presión durante la semana</t>
+          <t>Vigilar entradas en calle 12</t>
         </is>
       </c>
     </row>
@@ -1784,7 +2076,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>TRE-01</t>
+          <t>RCS-01</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -1794,7 +2086,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Chequeo de finales de carrera y lubricación de guías verticales.</t>
+          <t>Chequeo del rack de carga: tensiones por posición y ventilación normales.</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1828,7 +2120,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>TRK-03</t>
+          <t>CNV-01</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -1876,7 +2168,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>ETI-01</t>
+          <t>CLG-01</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1886,7 +2178,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>PM mensual: limpieza de cabezal, cambio de ribbon y prueba de aplicado.</t>
+          <t>PM mensual: limpieza de conectores, torque de bornes y prueba de carga.</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1904,7 +2196,7 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-07-10</t>
+          <t>OT-2026-07-18</t>
         </is>
       </c>
     </row>
@@ -1924,7 +2216,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-02</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1934,7 +2226,7 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Acompañamiento en peak de despacho, sin intervenciones.</t>
+          <t>Acompañamiento en peak de despacho, tráfico LGV sin intervenciones.</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1968,7 +2260,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>JOL-01</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -1978,7 +2270,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Lubricación de cadena de mesa giratoria y revisión de tensado.</t>
+          <t>Lubricación de cadenas de plataforma y revisión de nivel hidráulico.</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -2012,7 +2304,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>TRE-02</t>
+          <t>SAT-02</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -2022,7 +2314,7 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Reset y cambio de sensor de posición fina; transelevador quedó operativo.</t>
+          <t>Satélite atascado con pallet deforme en calle 8: rescate y prueba de ciclo.</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -2060,7 +2352,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>TRK-02</t>
+          <t>CNV-02</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -2070,7 +2362,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Revisión de empalmes de banda en muelle 5, se detecta desgaste leve.</t>
+          <t>Revisión de empalmes de banda en salida a andenes, desgaste leve.</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -2108,7 +2400,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>PAL-02</t>
+          <t>LGV-04</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -2118,7 +2410,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>PM mensual: revisión de ejes robot, torque de pernos base y respaldo de programa.</t>
+          <t>PM mensual: ruedas, frenos, scanner de seguridad y respaldo de parámetros.</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -2136,7 +2428,7 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-07-06</t>
+          <t>OT-2026-07-04</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2448,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>BSC-01</t>
+          <t>RCS-02</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -2166,7 +2458,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Verificación de calibración con pesas patrón, dentro de tolerancia.</t>
+          <t>Verificación de tensión de salida por posición de carga, en rango.</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -2200,7 +2492,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-03</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -2210,7 +2502,7 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Carro 214 con banda cortada: se reemplaza y se prueba en vacío.</t>
+          <t>LGV pierde localización en cruce C3: limpieza de reflectores y recalibración.</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -2248,17 +2540,17 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>ELE-01</t>
+          <t>SAT-01</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Inspección</t>
+          <t>Cambio de Batería</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Revisión de cadena de elevación y prueba de paradas de emergencia.</t>
+          <t>Cambio de batería y limpieza de contactos de carga del satélite.</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2292,7 +2584,7 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>TRK-01</t>
+          <t>CNV-01</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
@@ -2336,7 +2628,7 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>TRE-01</t>
+          <t>SAT-04</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -2346,7 +2638,7 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>PM mensual: inspección de cable de izaje, poleas y prueba de fin de pasillo.</t>
+          <t>PM mensual: baterías, sensórica, ruedas y prueba en calle vacía.</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2364,7 +2656,7 @@
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-07-07</t>
+          <t>OT-2026-07-09</t>
         </is>
       </c>
     </row>
@@ -2384,7 +2676,7 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-05</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
@@ -2394,7 +2686,7 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Limpieza profunda de lectores de código y espejos en inducciones 1-4.</t>
+          <t>Limpieza de scanner láser y ventanas de navegación de la flota LGV.</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -2428,7 +2720,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>JOL-01</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -2438,7 +2730,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Corte de film reiterado: se cambia porta-rollo dañado y se ajusta freno.</t>
+          <t>Cadena de arrastre con eslabón dañado: se reemplaza tramo y se prueba.</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2476,7 +2768,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>TRK-03</t>
+          <t>CNV-01</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -2486,7 +2778,7 @@
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Ronda general de transportadores, ruido anómalo en reductor E7.</t>
+          <t>Ronda general de conveyors, ruido anómalo en reductor E7.</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -2524,7 +2816,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>PAL-01</t>
+          <t>LGV-01</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -2534,7 +2826,7 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Supervisión armado de pallets mixtos, ajuste menor de mordaza.</t>
+          <t>Supervisión de tráfico LGV en peak, ajuste menor de prioridades en cruces.</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2568,7 +2860,7 @@
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>TRE-02</t>
+          <t>SAT-05</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
@@ -2578,7 +2870,7 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>PM mensual: lubricación de guías, revisión de shuttle y limpieza de sensórica.</t>
+          <t>PM mensual: baterías, limpieza de sensórica y prueba de ciclo completo.</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -2596,7 +2888,7 @@
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-07-08</t>
+          <t>OT-2026-07-10</t>
         </is>
       </c>
     </row>
@@ -2616,7 +2908,7 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>ETI-01</t>
+          <t>CLG-02</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -2626,7 +2918,7 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Reposicionamiento de aplicador: etiquetas quedaban dobladas en cajas bajas.</t>
+          <t>Reposicionamiento de guía de conector: el LGV no enganchaba al primer intento.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -2660,7 +2952,7 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>TRK-02</t>
+          <t>CNV-02</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
@@ -2670,7 +2962,7 @@
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>Cambio de banda desgastada en muelle 5 según pendiente del 22-07.</t>
+          <t>Cambio de banda desgastada en salida a andenes según pendiente del 22-07.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -2708,7 +3000,7 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-02</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -2718,7 +3010,7 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Chequeo de variadores en sala eléctrica, temperaturas normales.</t>
+          <t>Chequeo de variadores y temperaturas de tracción, normales.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -2752,7 +3044,7 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>ELE-01</t>
+          <t>SAT-03</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
@@ -2762,7 +3054,7 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Elevador detenido por cadena destensada, se tensa y verifica alineación.</t>
+          <t>Satélite detenido por batería agotada en calle: rescate y cambio de batería.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -2800,7 +3092,7 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>BSC-01</t>
+          <t>CLG-03</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -2810,7 +3102,7 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>PM mensual: limpieza de celda de carga y verificación con pesas patrón.</t>
+          <t>PM mensual: limpieza de conectores, torque de bornes y prueba de carga.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -2828,7 +3120,7 @@
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-07-11</t>
+          <t>OT-2026-07-20</t>
         </is>
       </c>
     </row>
@@ -2848,7 +3140,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>TRK-01</t>
+          <t>CNV-01</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
@@ -2892,7 +3184,7 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-04</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -2902,7 +3194,7 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Inducción 3 sin lectura: se reemplaza fotocelda de gatillo.</t>
+          <t>Scanner de seguridad con paradas falsas: limpieza y reemplazo de mica.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -2940,7 +3232,7 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>PAL-01</t>
+          <t>JOL-01</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
@@ -2950,7 +3242,7 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>PM mensual: revisión de reductores de ejes, engrase y respaldo de PLC.</t>
+          <t>PM mensual: plataforma, cadenas, presión hidráulica y prueba con camión vacío.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -2968,7 +3260,7 @@
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-07-05</t>
+          <t>OT-2026-07-15</t>
         </is>
       </c>
     </row>
@@ -2988,7 +3280,7 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>TRK-03</t>
+          <t>CNV-01</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -3036,7 +3328,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>TRE-01</t>
+          <t>SAT-06</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
@@ -3046,7 +3338,7 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>Ronda nocturna bodega automática, telemetría normal.</t>
+          <t>Ronda bodega de racks, telemetría de satélites normal.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -3080,7 +3372,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-03</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -3090,7 +3382,7 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>PM mensual sorter: revisión de carros, bandas, cadena principal y lubricación.</t>
+          <t>PM mensual: tracción, frenos, navegación y respaldo de configuración.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -3099,7 +3391,7 @@
         </is>
       </c>
       <c r="H33" s="7" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
@@ -3108,7 +3400,7 @@
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-07-01</t>
+          <t>OT-2026-07-03</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3420,7 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>SAT-07</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
@@ -3138,12 +3430,12 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Chequeo de mesa giratoria y sensor de altura de pallet.</t>
+          <t>Chequeo visual del satélite en calle; PM mensual sigue pendiente.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Operativa</t>
+          <t>Operativa con Observación</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -3151,10 +3443,14 @@
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J34" s="7" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>PM SAT-07 atrasada (OT-2026-07-12)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="n">
@@ -3172,7 +3468,7 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>TRK-02</t>
+          <t>CNV-02</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -3216,7 +3512,7 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>TRE-02</t>
+          <t>SAT-06</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
@@ -3226,7 +3522,7 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Transelevador B con alarma de sobrecarga: se recalibra celda y se libera.</t>
+          <t>Lecturas erráticas de posición: se recalibra encoder y queda en observación.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -3264,7 +3560,7 @@
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>TRK-01</t>
+          <t>CNV-01</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -3274,7 +3570,7 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Retiro de zunchos enredados en rodillos de recepción.</t>
+          <t>Retiro de zunchos enredados en rodillos de entrada.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -3308,7 +3604,7 @@
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>PAL-02</t>
+          <t>JOL-01</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
@@ -3318,7 +3614,7 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>Paletizador 2 detenido: colisión leve de garra, se revisa y reinicia con ajuste.</t>
+          <t>Plataforma pierde presión al cargar camión: fuga en central hidráulica.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -3336,7 +3632,7 @@
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
-          <t>Falla F-2026-039 abierta, esperando repuesto mordaza</t>
+          <t>Falla F-2026-039 abierta, esperando central hidráulica</t>
         </is>
       </c>
     </row>
@@ -3356,7 +3652,7 @@
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>PAL-02</t>
+          <t>JOL-01</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
@@ -3366,7 +3662,7 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Continúa intervención de garra; repuesto llega en la tarde.</t>
+          <t>Continúa cambio de central hidráulica; repuesto llega en la tarde.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -3404,7 +3700,7 @@
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-01</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
@@ -3414,7 +3710,7 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>Ronda de inicio de turno, parámetros normales tras PM de julio.</t>
+          <t>Ronda de inicio de turno: flota LGV y cruces sin novedades.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -3448,7 +3744,7 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>ETI-01</t>
+          <t>LGV-02</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -3458,7 +3754,7 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>PM mensual agosto: limpieza de cabezal y verificación de sensor de etiqueta.</t>
+          <t>PM mensual agosto: ruedas, scanner de seguridad y prueba de frenado.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -3467,7 +3763,7 @@
         </is>
       </c>
       <c r="H41" s="7" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
@@ -3476,7 +3772,7 @@
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-08-10</t>
+          <t>OT-2026-08-02</t>
         </is>
       </c>
     </row>
@@ -3493,7 +3789,7 @@
       <formula1>Maquinas!$A$2:$A$200</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Listas!$B$2:$B$10</formula1>
+      <formula1>Listas!$B$2:$B$11</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Listas!$C$2:$C$4</formula1>
@@ -3608,7 +3904,7 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-05</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
@@ -3628,7 +3924,7 @@
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>PLC pierde comunicación con scanner de inducción 2.</t>
+          <t>LGV pierde comunicación con el PLC de tráfico en zona de cruces.</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr">
@@ -3644,12 +3940,12 @@
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>Reinicio de switch y cambio de patch cord dañado.</t>
+          <t>Reinicio de AP wifi y cambio de antena dañada.</t>
         </is>
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>Patch cord Cat6</t>
+          <t>Antena wifi</t>
         </is>
       </c>
       <c r="M2" s="7" t="inlineStr">
@@ -3669,7 +3965,7 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>TRK-02</t>
+          <t>CNV-02</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
@@ -3689,7 +3985,7 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>Banda descentrada roza estructura en muelle 3.</t>
+          <t>Banda descentrada roza estructura en salida a andenes.</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
@@ -3726,7 +4022,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>TRE-01</t>
+          <t>SAT-04</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -3736,7 +4032,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Batería / Carga</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -3746,7 +4042,7 @@
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Variador de izaje dispara falla de sobrecorriente.</t>
+          <t>Satélite no inicia turno: batería sin carga tras la noche en el rack.</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
@@ -3762,12 +4058,12 @@
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>Cambio de ventilador de variador y limpieza de disipador.</t>
+          <t>Posición 3 del rack defectuosa: cambio de fusible y satélite a posición alterna.</t>
         </is>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
-          <t>Ventilador 24V</t>
+          <t>Fusible 63A</t>
         </is>
       </c>
       <c r="M4" s="7" t="inlineStr">
@@ -3787,7 +4083,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>ETI-01</t>
+          <t>LGV-05</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -3807,7 +4103,7 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Sensor de etiqueta con lecturas intermitentes.</t>
+          <t>Scanner de seguridad con lecturas intermitentes.</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
@@ -3823,7 +4119,7 @@
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Limpieza y reposicionamiento del sensor.</t>
+          <t>Limpieza y reposicionamiento de la mica del scanner.</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr"/>
@@ -3844,7 +4140,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>PAL-01</t>
+          <t>SAT-05</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -3854,7 +4150,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Neumática</t>
+          <t>Mecánica</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -3864,7 +4160,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Pérdida de vacío en ventosas de garra.</t>
+          <t>Rueda de rodadura con juego: el satélite vibra en la calle.</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -3880,12 +4176,12 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Cambio de manguera fisurada y regulación de presión.</t>
+          <t>Cambio de rueda y torque del eje.</t>
         </is>
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>Manguera PU 8mm</t>
+          <t>Rueda rodadura</t>
         </is>
       </c>
       <c r="M6" s="7" t="inlineStr">
@@ -3905,7 +4201,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-01</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -3925,7 +4221,7 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Atasco masivo por caja deformada en inducción 4.</t>
+          <t>Bloqueo de tráfico LGV por pallet mal dejado en cruce C2.</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -3941,7 +4237,7 @@
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>Despeje de línea y verificación de guías laterales.</t>
+          <t>Despeje del cruce y charla a operación.</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr"/>
@@ -3962,7 +4258,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>TRK-03</t>
+          <t>CNV-01</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -4023,7 +4319,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>TRE-02</t>
+          <t>SAT-02</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -4033,7 +4329,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Sensórica</t>
+          <t>Operacional</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -4043,7 +4339,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Transelevador B pierde posición fina en pasillo.</t>
+          <t>Satélite atascado con pallet deforme en calle 8.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -4059,14 +4355,10 @@
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>Cambio de sensor de posicionamiento y recalibración.</t>
-        </is>
-      </c>
-      <c r="L9" s="7" t="inlineStr">
-        <is>
-          <t>Sensor láser</t>
-        </is>
-      </c>
+          <t>Rescate del satélite, retiro del pallet y prueba de ciclo.</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr"/>
       <c r="M9" s="7" t="inlineStr">
         <is>
           <t>Miguel Ríos</t>
@@ -4084,7 +4376,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-03</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -4094,7 +4386,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Mecánica</t>
+          <t>Sensórica</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -4104,7 +4396,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Carro 214 con banda cortada, desvíos con error.</t>
+          <t>LGV pierde localización en cruce C3 y se detiene por seguridad.</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -4120,14 +4412,10 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>Reemplazo de banda de carro y prueba en vacío.</t>
-        </is>
-      </c>
-      <c r="L10" s="7" t="inlineStr">
-        <is>
-          <t>Banda cross-belt</t>
-        </is>
-      </c>
+          <t>Limpieza de reflectores y recalibración de navegación.</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr"/>
       <c r="M10" s="7" t="inlineStr">
         <is>
           <t>Rodrigo Pinto</t>
@@ -4145,7 +4433,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>JOL-01</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -4160,12 +4448,12 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Corte de film reiterado en inicio de ciclo.</t>
+          <t>Cadena de arrastre con eslabón dañado en plataforma.</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -4181,12 +4469,12 @@
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>Cambio de porta-rollo y ajuste de freno de film.</t>
+          <t>Reemplazo de tramo de cadena y prueba de ciclo.</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>Porta-rollo</t>
+          <t>Tramo cadena</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
@@ -4206,7 +4494,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>ELE-01</t>
+          <t>SAT-03</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -4216,7 +4504,7 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Mecánica</t>
+          <t>Batería / Carga</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -4226,7 +4514,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Elevador detenido: cadena destensada activa sensor de seguridad.</t>
+          <t>Satélite detenido en calle por batería agotada.</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -4242,10 +4530,14 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Tensado de cadena y verificación de alineación.</t>
-        </is>
-      </c>
-      <c r="L12" s="7" t="inlineStr"/>
+          <t>Rescate, cambio de batería y revisión de contactos.</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>Batería 24V</t>
+        </is>
+      </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
           <t>Rodrigo Pinto</t>
@@ -4263,7 +4555,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-04</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -4283,7 +4575,7 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Inducción 3 sin lectura de paquetes.</t>
+          <t>Scanner de seguridad genera paradas falsas en pasillo.</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -4299,12 +4591,12 @@
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>Reemplazo de fotocelda de gatillo.</t>
+          <t>Limpieza profunda y reemplazo de mica rayada.</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>Fotocelda difusa</t>
+          <t>Mica scanner</t>
         </is>
       </c>
       <c r="M13" s="7" t="inlineStr">
@@ -4324,7 +4616,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>TRK-03</t>
+          <t>CNV-01</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -4385,7 +4677,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>TRE-02</t>
+          <t>SAT-06</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -4395,7 +4687,7 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Sensórica</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -4405,7 +4697,7 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Alarma de sobrecarga en izaje al tomar pallets pesados.</t>
+          <t>Lecturas erráticas de posición dentro del rack.</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -4419,7 +4711,7 @@
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>Recalibración de celda de carga; en observación 72 h.</t>
+          <t>Recalibración de encoder; en observación 72 h.</t>
         </is>
       </c>
       <c r="L15" s="7" t="inlineStr"/>
@@ -4440,7 +4732,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>PAL-02</t>
+          <t>JOL-01</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -4450,7 +4742,7 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Mecánica</t>
+          <t>Hidráulica</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
@@ -4460,7 +4752,7 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Colisión de garra con pallet mal posicionado; mordaza dañada.</t>
+          <t>Plataforma pierde presión al cargar camión: fuga en central hidráulica.</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
@@ -4474,12 +4766,12 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>A la espera de repuesto de mordaza (llega 02-08 tarde).</t>
+          <t>A la espera de central hidráulica (llega 02-08 en la tarde).</t>
         </is>
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>Mordaza garra</t>
+          <t>Central hidráulica</t>
         </is>
       </c>
       <c r="M16" s="7" t="inlineStr">
@@ -4499,7 +4791,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>TRK-01</t>
+          <t>CNV-01</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -4519,7 +4811,7 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Zunchos enredados detienen rodillos de recepción.</t>
+          <t>Zunchos enredados detienen rodillos de entrada.</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -4555,7 +4847,7 @@
       <formula1>Listas!$A$2:$A$4</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Listas!$D$2:$D$7</formula1>
+      <formula1>Listas!$D$2:$D$8</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Listas!$E$2:$E$5</formula1>
@@ -4577,7 +4869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4652,12 +4944,12 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>LGV-01</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Revisión de carros, bandas, cadena principal y lubricación general</t>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
@@ -4666,10 +4958,10 @@
         </is>
       </c>
       <c r="E2" s="9" t="n">
-        <v>46234</v>
+        <v>46210</v>
       </c>
       <c r="F2" s="9" t="n">
-        <v>46234</v>
+        <v>46210</v>
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
@@ -4678,11 +4970,11 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>Javiera Soto</t>
+          <t>Carlos Bravo</t>
         </is>
       </c>
       <c r="I2" s="7" t="n">
-        <v>240</v>
+        <v>90</v>
       </c>
       <c r="J2" s="7" t="inlineStr"/>
     </row>
@@ -4694,12 +4986,12 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>TRK-01</t>
+          <t>LGV-02</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Inspección de rodillos, bandas y motorreductores; limpieza de sensórica</t>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
@@ -4708,10 +5000,10 @@
         </is>
       </c>
       <c r="E3" s="9" t="n">
-        <v>46218</v>
+        <v>46211</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>46218</v>
+        <v>46211</v>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
@@ -4720,11 +5012,11 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Miguel Ríos</t>
+          <t>Constanza Díaz</t>
         </is>
       </c>
       <c r="I3" s="7" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="J3" s="7" t="inlineStr"/>
     </row>
@@ -4736,12 +5028,12 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>TRK-02</t>
+          <t>LGV-03</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Inspección de rodillos, bandas y motorreductores; limpieza de sensórica</t>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -4750,10 +5042,10 @@
         </is>
       </c>
       <c r="E4" s="9" t="n">
-        <v>46219</v>
+        <v>46234</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>46221</v>
+        <v>46234</v>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
@@ -4762,17 +5054,13 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Miguel Ríos</t>
+          <t>Javiera Soto</t>
         </is>
       </c>
       <c r="I4" s="7" t="n">
-        <v>75</v>
-      </c>
-      <c r="J4" s="7" t="inlineStr">
-        <is>
-          <t>Se corrió 2 días por peak de despacho</t>
-        </is>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="J4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -4782,12 +5070,12 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>TRK-03</t>
+          <t>LGV-04</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Inspección de rodillos, bandas y motorreductores; limpieza de sensórica</t>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -4796,10 +5084,10 @@
         </is>
       </c>
       <c r="E5" s="9" t="n">
-        <v>46220</v>
+        <v>46226</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>46220</v>
+        <v>46226</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -4808,11 +5096,11 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Felipe Aravena</t>
+          <t>Carlos Bravo</t>
         </is>
       </c>
       <c r="I5" s="7" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="J5" s="7" t="inlineStr"/>
     </row>
@@ -4824,12 +5112,12 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>PAL-01</t>
+          <t>LGV-05</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Revisión de reductores de ejes, engrase, torque y respaldo de PLC</t>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -4838,10 +5126,10 @@
         </is>
       </c>
       <c r="E6" s="9" t="n">
-        <v>46233</v>
+        <v>46213</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>46233</v>
+        <v>46213</v>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
@@ -4850,11 +5138,11 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Carlos Bravo</t>
+          <t>Miguel Ríos</t>
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="J6" s="7" t="inlineStr"/>
     </row>
@@ -4866,12 +5154,12 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>PAL-02</t>
+          <t>SAT-01</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Revisión de reductores de ejes, engrase, torque y respaldo de PLC</t>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -4880,10 +5168,10 @@
         </is>
       </c>
       <c r="E7" s="9" t="n">
-        <v>46226</v>
+        <v>46216</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>46226</v>
+        <v>46216</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -4892,11 +5180,11 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Carlos Bravo</t>
+          <t>Javiera Soto</t>
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="J7" s="7" t="inlineStr"/>
     </row>
@@ -4908,12 +5196,12 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>TRE-01</t>
+          <t>SAT-02</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Inspección de cable de izaje, poleas, guías y prueba de seguridad</t>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -4922,10 +5210,10 @@
         </is>
       </c>
       <c r="E8" s="9" t="n">
-        <v>46227</v>
+        <v>46217</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>46227</v>
+        <v>46217</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -4934,11 +5222,11 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Felipe Aravena</t>
+          <t>Miguel Ríos</t>
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="J8" s="7" t="inlineStr"/>
     </row>
@@ -4950,12 +5238,12 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>TRE-02</t>
+          <t>SAT-03</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Lubricación de guías, revisión de shuttle y limpieza de sensórica</t>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -4964,10 +5252,10 @@
         </is>
       </c>
       <c r="E9" s="9" t="n">
-        <v>46230</v>
+        <v>46218</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>46230</v>
+        <v>46218</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
@@ -4976,11 +5264,11 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Javiera Soto</t>
+          <t>Rodrigo Pinto</t>
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="J9" s="7" t="inlineStr"/>
     </row>
@@ -4992,12 +5280,12 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>SAT-04</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Revisión de mesa giratoria, cadena, freno de film y sensores</t>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -5006,24 +5294,25 @@
         </is>
       </c>
       <c r="E10" s="9" t="n">
-        <v>46225</v>
-      </c>
-      <c r="F10" s="12" t="n"/>
+        <v>46227</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>46227</v>
+      </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Reprogramada</t>
+          <t>Realizada</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Constanza Díaz</t>
-        </is>
-      </c>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>Reprogramada al 05-08 por falta de repuesto</t>
-        </is>
-      </c>
+          <t>Felipe Aravena</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="J10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -5033,12 +5322,12 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>ETI-01</t>
+          <t>SAT-05</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Limpieza de cabezal, cambio de ribbon y prueba de aplicado</t>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -5047,10 +5336,10 @@
         </is>
       </c>
       <c r="E11" s="9" t="n">
-        <v>46224</v>
+        <v>46230</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>46224</v>
+        <v>46230</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
@@ -5059,11 +5348,11 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>Constanza Díaz</t>
+          <t>Javiera Soto</t>
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>40</v>
+        <v>140</v>
       </c>
       <c r="J11" s="7" t="inlineStr"/>
     </row>
@@ -5075,12 +5364,12 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>BSC-01</t>
+          <t>SAT-06</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Limpieza de celda de carga y verificación con pesas patrón</t>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -5089,10 +5378,10 @@
         </is>
       </c>
       <c r="E12" s="9" t="n">
-        <v>46232</v>
+        <v>46220</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>46232</v>
+        <v>46220</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
@@ -5101,11 +5390,11 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Javiera Soto</t>
+          <t>Felipe Aravena</t>
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="J12" s="7" t="inlineStr"/>
     </row>
@@ -5117,12 +5406,12 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>ELE-01</t>
+          <t>SAT-07</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Revisión y tensado de cadena de elevación, prueba de emergencias</t>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -5131,7 +5420,7 @@
         </is>
       </c>
       <c r="E13" s="9" t="n">
-        <v>46231</v>
+        <v>46228</v>
       </c>
       <c r="F13" s="12" t="n"/>
       <c r="G13" s="7" t="inlineStr">
@@ -5153,17 +5442,17 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-08-01</t>
+          <t>OT-2026-07-13</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>SOR-01</t>
+          <t>CNV-01</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Revisión de carros, bandas, cadena principal y lubricación general</t>
+          <t>Inspección de rodillos, bandas y motorreductores; limpieza de sensórica</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -5172,30 +5461,35 @@
         </is>
       </c>
       <c r="E14" s="9" t="n">
-        <v>46262</v>
-      </c>
-      <c r="F14" s="12" t="n"/>
+        <v>46223</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>46223</v>
+      </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Realizada</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Javiera Soto</t>
-        </is>
+          <t>Miguel Ríos</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>70</v>
       </c>
       <c r="J14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-08-02</t>
+          <t>OT-2026-07-14</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>TRK-01</t>
+          <t>CNV-02</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -5209,12 +5503,14 @@
         </is>
       </c>
       <c r="E15" s="9" t="n">
-        <v>46246</v>
-      </c>
-      <c r="F15" s="12" t="n"/>
+        <v>46219</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>46221</v>
+      </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Realizada</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -5222,22 +5518,29 @@
           <t>Miguel Ríos</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr"/>
+      <c r="I15" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>Se corrió 2 días por peak de despacho</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-08-03</t>
+          <t>OT-2026-07-15</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>TRK-02</t>
+          <t>JOL-01</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Inspección de rodillos, bandas y motorreductores; limpieza de sensórica</t>
+          <t>Revisión de plataforma, cadenas de arrastre y presión del sistema hidráulico</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -5246,35 +5549,40 @@
         </is>
       </c>
       <c r="E16" s="9" t="n">
-        <v>46247</v>
-      </c>
-      <c r="F16" s="12" t="n"/>
+        <v>46233</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>46233</v>
+      </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Realizada</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Miguel Ríos</t>
-        </is>
+          <t>Carlos Bravo</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>95</v>
       </c>
       <c r="J16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-08-04</t>
+          <t>OT-2026-07-16</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>TRK-03</t>
+          <t>RCS-01</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Inspección de rodillos, bandas y motorreductores; limpieza de sensórica</t>
+          <t>Limpieza de conectores, prueba de tensión por posición y revisión de ventilación</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -5283,35 +5591,39 @@
         </is>
       </c>
       <c r="E17" s="9" t="n">
-        <v>46248</v>
+        <v>46225</v>
       </c>
       <c r="F17" s="12" t="n"/>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Reprogramada</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Felipe Aravena</t>
-        </is>
-      </c>
-      <c r="J17" s="7" t="inlineStr"/>
+          <t>Constanza Díaz</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>Reprogramada al 05-08 por falta de ventilador</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-08-05</t>
+          <t>OT-2026-07-17</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>PAL-01</t>
+          <t>RCS-02</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Revisión de reductores de ejes, engrase, torque y respaldo de PLC</t>
+          <t>Limpieza de conectores, prueba de tensión por posición y revisión de ventilación</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -5320,35 +5632,44 @@
         </is>
       </c>
       <c r="E18" s="9" t="n">
-        <v>46260</v>
-      </c>
-      <c r="F18" s="12" t="n"/>
+        <v>46225</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>46227</v>
+      </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Realizada</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>Carlos Bravo</t>
-        </is>
-      </c>
-      <c r="J18" s="7" t="inlineStr"/>
+          <t>Constanza Díaz</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>Se corrió 2 días por disponibilidad de sala</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-08-06</t>
+          <t>OT-2026-07-18</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>PAL-02</t>
+          <t>CLG-01</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Revisión de reductores de ejes, engrase, torque y respaldo de PLC</t>
+          <t>Limpieza de conectores, torque de bornes y prueba de carga completa</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -5357,35 +5678,40 @@
         </is>
       </c>
       <c r="E19" s="9" t="n">
-        <v>46254</v>
-      </c>
-      <c r="F19" s="12" t="n"/>
+        <v>46224</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>46224</v>
+      </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Realizada</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>Carlos Bravo</t>
-        </is>
+          <t>Constanza Díaz</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>40</v>
       </c>
       <c r="J19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-08-07</t>
+          <t>OT-2026-07-19</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>TRE-01</t>
+          <t>CLG-02</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Inspección de cable de izaje, poleas, guías y prueba de seguridad</t>
+          <t>Limpieza de conectores, torque de bornes y prueba de carga completa</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -5394,7 +5720,7 @@
         </is>
       </c>
       <c r="E20" s="9" t="n">
-        <v>46255</v>
+        <v>46231</v>
       </c>
       <c r="F20" s="12" t="n"/>
       <c r="G20" s="7" t="inlineStr">
@@ -5404,25 +5730,29 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>Felipe Aravena</t>
-        </is>
-      </c>
-      <c r="J20" s="7" t="inlineStr"/>
+          <t>Miguel Ríos</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>No ejecutada: técnico derivado a falla de CNV-01</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-08-08</t>
+          <t>OT-2026-07-20</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>TRE-02</t>
+          <t>CLG-03</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Lubricación de guías, revisión de shuttle y limpieza de sensórica</t>
+          <t>Limpieza de conectores, torque de bornes y prueba de carga completa</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -5431,35 +5761,40 @@
         </is>
       </c>
       <c r="E21" s="9" t="n">
-        <v>46258</v>
-      </c>
-      <c r="F21" s="12" t="n"/>
+        <v>46232</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>46232</v>
+      </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Realizada</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
           <t>Javiera Soto</t>
         </is>
+      </c>
+      <c r="I21" s="7" t="n">
+        <v>45</v>
       </c>
       <c r="J21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-08-09</t>
+          <t>OT-2026-08-01</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>ENV-01</t>
+          <t>LGV-01</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Revisión de mesa giratoria, cadena, freno de film y sensores</t>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -5468,7 +5803,7 @@
         </is>
       </c>
       <c r="E22" s="9" t="n">
-        <v>46239</v>
+        <v>46244</v>
       </c>
       <c r="F22" s="12" t="n"/>
       <c r="G22" s="7" t="inlineStr">
@@ -5478,7 +5813,7 @@
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>Constanza Díaz</t>
+          <t>Carlos Bravo</t>
         </is>
       </c>
       <c r="J22" s="7" t="inlineStr"/>
@@ -5486,17 +5821,17 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-08-10</t>
+          <t>OT-2026-08-02</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>ETI-01</t>
+          <t>LGV-02</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Limpieza de cabezal, cambio de ribbon y prueba de aplicado</t>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -5521,24 +5856,24 @@
         </is>
       </c>
       <c r="I23" s="7" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="J23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-08-11</t>
+          <t>OT-2026-08-03</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>ELE-01</t>
+          <t>LGV-03</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Revisión y tensado de cadena de elevación, prueba de emergencias</t>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -5547,7 +5882,7 @@
         </is>
       </c>
       <c r="E24" s="9" t="n">
-        <v>46240</v>
+        <v>46262</v>
       </c>
       <c r="F24" s="12" t="n"/>
       <c r="G24" s="7" t="inlineStr">
@@ -5557,29 +5892,25 @@
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>Rodrigo Pinto</t>
-        </is>
-      </c>
-      <c r="J24" s="7" t="inlineStr">
-        <is>
-          <t>Incluye pendiente de julio</t>
-        </is>
-      </c>
+          <t>Javiera Soto</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>OT-2026-08-12</t>
+          <t>OT-2026-08-04</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>BSC-01</t>
+          <t>LGV-04</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Limpieza de celda de carga y verificación con pesas patrón</t>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -5588,7 +5919,7 @@
         </is>
       </c>
       <c r="E25" s="9" t="n">
-        <v>46261</v>
+        <v>46258</v>
       </c>
       <c r="F25" s="12" t="n"/>
       <c r="G25" s="7" t="inlineStr">
@@ -5598,10 +5929,614 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
+          <t>Carlos Bravo</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-05</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>LGV-05</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>46245</v>
+      </c>
+      <c r="F26" s="12" t="n"/>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Miguel Ríos</t>
+        </is>
+      </c>
+      <c r="J26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-06</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>SAT-01</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>46246</v>
+      </c>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
           <t>Javiera Soto</t>
         </is>
       </c>
-      <c r="J25" s="7" t="inlineStr"/>
+      <c r="J27" s="7" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-07</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>SAT-02</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>46247</v>
+      </c>
+      <c r="F28" s="12" t="n"/>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Miguel Ríos</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-08</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>SAT-03</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>46248</v>
+      </c>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Rodrigo Pinto</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-09</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>SAT-04</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>46259</v>
+      </c>
+      <c r="F30" s="12" t="n"/>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Felipe Aravena</t>
+        </is>
+      </c>
+      <c r="J30" s="7" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-10</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>SAT-05</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>46260</v>
+      </c>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Javiera Soto</t>
+        </is>
+      </c>
+      <c r="J31" s="7" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-11</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>SAT-06</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>46251</v>
+      </c>
+      <c r="F32" s="12" t="n"/>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Felipe Aravena</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-12</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>SAT-07</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas de rodadura y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>46240</v>
+      </c>
+      <c r="F33" s="12" t="n"/>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Rodrigo Pinto</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>Incluye pendiente de julio</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-13</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>CNV-01</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Inspección de rodillos, bandas y motorreductores; limpieza de sensórica</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>46238</v>
+      </c>
+      <c r="F34" s="12" t="n"/>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Miguel Ríos</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-14</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>CNV-02</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Inspección de rodillos, bandas y motorreductores; limpieza de sensórica</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>46252</v>
+      </c>
+      <c r="F35" s="12" t="n"/>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Miguel Ríos</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-15</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>JOL-01</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de plataforma, cadenas de arrastre y presión del sistema hidráulico</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="n">
+        <v>46261</v>
+      </c>
+      <c r="F36" s="12" t="n"/>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Carlos Bravo</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-16</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>RCS-01</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores, prueba de tensión por posición y revisión de ventilación</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="n">
+        <v>46239</v>
+      </c>
+      <c r="F37" s="12" t="n"/>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Constanza Díaz</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>Reprogramada de julio</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-17</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>RCS-02</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores, prueba de tensión por posición y revisión de ventilación</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="n">
+        <v>46253</v>
+      </c>
+      <c r="F38" s="12" t="n"/>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Constanza Díaz</t>
+        </is>
+      </c>
+      <c r="J38" s="7" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-18</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>CLG-01</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores, torque de bornes y prueba de carga completa</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="n">
+        <v>46254</v>
+      </c>
+      <c r="F39" s="12" t="n"/>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Constanza Díaz</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-19</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>CLG-02</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores, torque de bornes y prueba de carga completa</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>46241</v>
+      </c>
+      <c r="F40" s="12" t="n"/>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Miguel Ríos</t>
+        </is>
+      </c>
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t>Incluye pendiente de julio</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>OT-2026-08-20</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>CLG-03</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores, torque de bornes y prueba de carga completa</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="n">
+        <v>46265</v>
+      </c>
+      <c r="F41" s="12" t="n"/>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Javiera Soto</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>

</xml_diff>

<commit_message>
Agrega pautas por equipo, plan multi-frecuencia y arquitectura de integración
Nueva pestaña Pautas en la plantilla (100 pautas: 20 equipos x 5
frecuencias diaria/semanal/mensual/semestral/anual) con link al documento
del fabricante, su consulta Power Query en ambos métodos y la relación en
el modelo. La guía suma la página de pautas segmentada por fabricante, la
tabla de dónde vive cada frecuencia del plan y la ficha por equipo con
obtención de detalles (drillthrough) que enlaza bitácora, fallas, pautas e
historial. Documenta la hoja de ruta de integración en fases con el
software de la empresa (Power Automate, Azure, Snowflake) en
docs/ARQUITECTURA_INTEGRACION.md.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VZDcZPRf2zrYzCo4cb6M6C
</commit_message>
<xml_diff>
--- a/powerbi-mantencion/plantilla/Plantilla_Bitacora_Mantencion.xlsx
+++ b/powerbi-mantencion/plantilla/Plantilla_Bitacora_Mantencion.xlsx
@@ -13,12 +13,14 @@
     <sheet name="Bitacora" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Fallas" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="MantencionMensual" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Pautas" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Maquinas'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Bitacora'!$A$1:$J$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Fallas'!$A$1:$M$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'MantencionMensual'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Pautas'!$A$1:$G$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -490,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E23"/>
+  <dimension ref="B2:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -610,7 +612,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Catálogo de equipos: ID, nombre, zona, criticidad</t>
+          <t>Catálogo de equipos: ID, nombre, sección, zona, criticidad y fabricante</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -627,100 +629,122 @@
     <row r="10" ht="34" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
+          <t>Pautas</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Pauta de mantención de cada equipo por frecuencia (diaria a anual), con link al documento del fabricante</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Al definir o actualizar pautas</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
           <t>Listas</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Valores válidos de los desplegables (técnicos, turnos, estados…)</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Supervisor</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Solo cuando cambie el equipo de trabajo</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="6" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>REGLAS DE USO</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>1. Fechas en formato AAAA-MM-DD (ej: 2026-08-02) y fecha-hora como AAAA-MM-DD HH:MM. Las columnas ya vienen con ese formato.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>2. Detencion_Min y Duracion_Min siempre en minutos enteros (ej: 90, no "1,5 h").</t>
+          <t>1. Fechas en formato AAAA-MM-DD (ej: 2026-08-02) y fecha-hora como AAAA-MM-DD HH:MM. Las columnas ya vienen con ese formato.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>3. Usar los desplegables de cada columna; si falta un técnico o un valor, agregarlo primero en la pestaña Listas.</t>
+          <t>2. Detencion_Min y Duracion_Min siempre en minutos enteros (ej: 90, no "1,5 h").</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>4. Una fila por actividad o falla. No dejar filas en blanco entre registros ni combinar celdas.</t>
+          <t>3. Usar los desplegables de cada columna; si falta un técnico o un valor, agregarlo primero en la pestaña Listas.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>5. Una falla que sigue abierta al cambio de turno se deja con Estado "Abierta" o "En Reparación" y sin Fecha_Hora_Cierre.</t>
+          <t>4. Una fila por actividad o falla. No dejar filas en blanco entre registros ni combinar celdas.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="7" t="inlineStr">
         <is>
+          <t>5. Una falla que sigue abierta al cambio de turno se deja con Estado "Abierta" o "En Reparación" y sin Fecha_Hora_Cierre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
           <t>6. Las filas actuales son EJEMPLOS para probar el dashboard: bórrelas cuando empiecen a registrar datos reales (deje los encabezados).</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="7" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>CÓMO SUBIRLA A GOOGLE SHEETS</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>1. En Google Drive: Nuevo → Subir archivo → seleccionar este Excel.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>2. Abrir con Google Sheets y usar Archivo → Guardar como hoja de cálculo de Google.</t>
+          <t>1. En Google Drive: Nuevo → Subir archivo → seleccionar este Excel.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>2. Abrir con Google Sheets y usar Archivo → Guardar como hoja de cálculo de Google.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>3. Compartir con el equipo (editores) y conectar Power BI según la guía del repositorio (carpeta docs/).</t>
         </is>
@@ -848,7 +872,7 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>Mensual</t>
+          <t>Diaria</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
@@ -905,7 +929,7 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Bimestral</t>
+          <t>Semanal</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
@@ -962,7 +986,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Trimestral</t>
+          <t>Mensual</t>
         </is>
       </c>
       <c r="J4" s="7" t="inlineStr">
@@ -999,7 +1023,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Semestral</t>
+          <t>Bimestral</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
@@ -1021,7 +1045,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Anual</t>
+          <t>Trimestral</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
@@ -1041,6 +1065,11 @@
           <t>Batería / Carga</t>
         </is>
       </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
           <t>Rodrigo Pinto</t>
@@ -1056,6 +1085,11 @@
       <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Operacional</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
         </is>
       </c>
     </row>
@@ -6545,7 +6579,7 @@
       <formula1>Maquinas!$A$2:$A$200</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Listas!$H$2:$H$6</formula1>
+      <formula1>Listas!$H$2:$H$8</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Listas!$G$2:$G$5</formula1>
@@ -6556,4 +6590,3573 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G101"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>ID_Pauta</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>ID_Maquina</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Frecuencia</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Duracion_Min_Est</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Link_Pauta</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-01-D</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>LGV-01</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Chequeo visual, limpieza de scanner y prueba de frenos al inicio de turno</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-01-S</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>LGV-01</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de reflectores y revisión de desgaste de ruedas</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-01-M</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>LGV-01</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-01-SE</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>LGV-01</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de ruedas según desgaste, revisión de tracción y calibración láser</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-01-A</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>LGV-01</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Overhaul según pauta del fabricante: tracción, baterías y sistemas de seguridad</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>480</v>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-02-D</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>LGV-02</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Chequeo visual, limpieza de scanner y prueba de frenos al inicio de turno</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-02-S</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>LGV-02</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de reflectores y revisión de desgaste de ruedas</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-02-M</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>LGV-02</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-02-SE</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>LGV-02</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de ruedas según desgaste, revisión de tracción y calibración láser</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-02-A</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>LGV-02</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Overhaul según pauta del fabricante: tracción, baterías y sistemas de seguridad</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>480</v>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-03-D</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>LGV-03</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Chequeo visual, limpieza de scanner y prueba de frenos al inicio de turno</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-03-S</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>LGV-03</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de reflectores y revisión de desgaste de ruedas</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-03-M</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>LGV-03</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-03-SE</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>LGV-03</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de ruedas según desgaste, revisión de tracción y calibración láser</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-03-A</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>LGV-03</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Overhaul según pauta del fabricante: tracción, baterías y sistemas de seguridad</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>480</v>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-04-D</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>LGV-04</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Chequeo visual, limpieza de scanner y prueba de frenos al inicio de turno</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-04-S</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>LGV-04</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de reflectores y revisión de desgaste de ruedas</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-04-M</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>LGV-04</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-04-SE</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>LGV-04</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de ruedas según desgaste, revisión de tracción y calibración láser</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-04-A</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>LGV-04</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Overhaul según pauta del fabricante: tracción, baterías y sistemas de seguridad</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>480</v>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-05-D</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>LGV-05</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Chequeo visual, limpieza de scanner y prueba de frenos al inicio de turno</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-05-S</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>LGV-05</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de reflectores y revisión de desgaste de ruedas</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-05-M</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>LGV-05</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de ruedas, frenos, scanner de seguridad, navegación y respaldo de parámetros</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-05-SE</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>LGV-05</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de ruedas según desgaste, revisión de tracción y calibración láser</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>P-LGV-05-A</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>LGV-05</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Overhaul según pauta del fabricante: tracción, baterías y sistemas de seguridad</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>480</v>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-01-D</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>SAT-01</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Chequeo de batería y contactos de carga al inicio de turno</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-01-S</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>SAT-01</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de sensórica y revisión de ruedas de rodadura</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-01-M</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>SAT-01</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-01-SE</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>SAT-01</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de baterías/ruedas según estado y calibración de encoder</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-01-A</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>SAT-01</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Overhaul según pauta del fabricante</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-02-D</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>SAT-02</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Chequeo de batería y contactos de carga al inicio de turno</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-02-S</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>SAT-02</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de sensórica y revisión de ruedas de rodadura</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-02-M</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>SAT-02</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-02-SE</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>SAT-02</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de baterías/ruedas según estado y calibración de encoder</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-02-A</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>SAT-02</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Overhaul según pauta del fabricante</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-03-D</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>SAT-03</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Chequeo de batería y contactos de carga al inicio de turno</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-03-S</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>SAT-03</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de sensórica y revisión de ruedas de rodadura</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-03-M</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>SAT-03</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-03-SE</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>SAT-03</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de baterías/ruedas según estado y calibración de encoder</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-03-A</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>SAT-03</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Overhaul según pauta del fabricante</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-04-D</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>SAT-04</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Chequeo de batería y contactos de carga al inicio de turno</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-04-S</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>SAT-04</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de sensórica y revisión de ruedas de rodadura</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-04-M</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>SAT-04</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-04-SE</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>SAT-04</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de baterías/ruedas según estado y calibración de encoder</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-04-A</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>SAT-04</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Overhaul según pauta del fabricante</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-05-D</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>SAT-05</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Chequeo de batería y contactos de carga al inicio de turno</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-05-S</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>SAT-05</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de sensórica y revisión de ruedas de rodadura</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-05-M</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>SAT-05</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-05-SE</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>SAT-05</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de baterías/ruedas según estado y calibración de encoder</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-05-A</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>SAT-05</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Overhaul según pauta del fabricante</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-06-D</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>SAT-06</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Chequeo de batería y contactos de carga al inicio de turno</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-06-S</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>SAT-06</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de sensórica y revisión de ruedas de rodadura</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-06-M</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>SAT-06</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-06-SE</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>SAT-06</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de baterías/ruedas según estado y calibración de encoder</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-06-A</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>SAT-06</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Overhaul según pauta del fabricante</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-07-D</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>SAT-07</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Chequeo de batería y contactos de carga al inicio de turno</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-07-S</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>SAT-07</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de sensórica y revisión de ruedas de rodadura</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-07-M</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>SAT-07</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de baterías, sensórica, ruedas y prueba de ciclo completo</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-07-SE</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>SAT-07</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de baterías/ruedas según estado y calibración de encoder</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="n">
+        <v>210</v>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>P-SAT-07-A</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>SAT-07</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>Overhaul según pauta del fabricante</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-AUTOMHA</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>P-CNV-01-D</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>CNV-01</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>Ronda visual: rodillos, bandas y fotoceldas</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-INTERROLL</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>P-CNV-01-S</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>CNV-01</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de fotoceldas y revisión de tensado de bandas</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-INTERROLL</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>P-CNV-01-M</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>CNV-01</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>Inspección de rodillos, bandas y motorreductores; limpieza de sensórica</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-INTERROLL</t>
+        </is>
+      </c>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>P-CNV-01-SE</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>CNV-01</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de rodamientos y bandas según desgaste</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-INTERROLL</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>P-CNV-01-A</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>CNV-01</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>Revisión mayor de estructura, motorreductores y tableros eléctricos</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="F66" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-INTERROLL</t>
+        </is>
+      </c>
+      <c r="G66" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>P-CNV-02-D</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>CNV-02</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>Ronda visual: rodillos, bandas y fotoceldas</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-INTERROLL</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>P-CNV-02-S</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>CNV-02</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de fotoceldas y revisión de tensado de bandas</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-INTERROLL</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>P-CNV-02-M</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>CNV-02</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>Inspección de rodillos, bandas y motorreductores; limpieza de sensórica</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-INTERROLL</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>P-CNV-02-SE</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>CNV-02</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de rodamientos y bandas según desgaste</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-INTERROLL</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>P-CNV-02-A</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>CNV-02</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>Revisión mayor de estructura, motorreductores y tableros eléctricos</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-INTERROLL</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>P-JOL-01-D</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>JOL-01</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Chequeo de presión hidráulica y prueba de plataforma en vacío</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-JOLODA</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>P-JOL-01-S</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>JOL-01</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>Lubricación de cadenas de arrastre y revisión de nivel hidráulico</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-JOLODA</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>P-JOL-01-M</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>JOL-01</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>Revisión de plataforma, cadenas y presión del sistema hidráulico</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="n">
+        <v>95</v>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-JOLODA</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>P-JOL-01-SE</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>JOL-01</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>Cambio de aceite hidráulico y revisión de sellos</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-JOLODA</t>
+        </is>
+      </c>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>P-JOL-01-A</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>JOL-01</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Overhaul según pauta del fabricante</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="n">
+        <v>480</v>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-JOLODA</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>P-RCS-01-D</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>RCS-01</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Verificación rápida de estados y alarmas del rack</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-FRONIUS</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>P-RCS-01-S</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>RCS-01</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores y chequeo visual de ventilación</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-FRONIUS</t>
+        </is>
+      </c>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>P-RCS-01-M</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>RCS-01</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores, prueba de tensión por posición y ventilación</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-FRONIUS</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>P-RCS-01-SE</t>
+        </is>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>RCS-01</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>Revisión termográfica de conexiones</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="F80" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-FRONIUS</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>P-RCS-01-A</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>RCS-01</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>Mantención eléctrica mayor certificada</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-FRONIUS</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>P-RCS-02-D</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>RCS-02</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>Verificación rápida de estados y alarmas del rack</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-FRONIUS</t>
+        </is>
+      </c>
+      <c r="G82" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="7" t="inlineStr">
+        <is>
+          <t>P-RCS-02-S</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>RCS-02</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores y chequeo visual de ventilación</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-FRONIUS</t>
+        </is>
+      </c>
+      <c r="G83" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>P-RCS-02-M</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>RCS-02</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores, prueba de tensión por posición y ventilación</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="F84" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-FRONIUS</t>
+        </is>
+      </c>
+      <c r="G84" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>P-RCS-02-SE</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>RCS-02</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>Revisión termográfica de conexiones</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-FRONIUS</t>
+        </is>
+      </c>
+      <c r="G85" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>P-RCS-02-A</t>
+        </is>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>RCS-02</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="inlineStr">
+        <is>
+          <t>Mantención eléctrica mayor certificada</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="F86" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-FRONIUS</t>
+        </is>
+      </c>
+      <c r="G86" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-01-D</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>CLG-01</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t>Verificación rápida de estados y alarmas del cargador</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G87" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-01-S</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>CLG-01</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores y chequeo visual de ventilación</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F88" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G88" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-01-M</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>CLG-01</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores, torque de bornes y prueba de carga completa</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G89" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-01-SE</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>CLG-01</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="inlineStr">
+        <is>
+          <t>Revisión termográfica de conexiones</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="F90" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G90" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-01-A</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>CLG-01</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
+          <t>Mantención eléctrica mayor certificada</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="F91" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G91" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-02-D</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>CLG-02</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>Verificación rápida de estados y alarmas del cargador</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G92" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-02-S</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>CLG-02</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D93" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores y chequeo visual de ventilación</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F93" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G93" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-02-M</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>CLG-02</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores, torque de bornes y prueba de carga completa</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G94" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-02-SE</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>CLG-02</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>Revisión termográfica de conexiones</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G95" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-02-A</t>
+        </is>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
+        <is>
+          <t>CLG-02</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t>Mantención eléctrica mayor certificada</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="F96" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G96" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-03-D</t>
+        </is>
+      </c>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>CLG-03</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>Diaria</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>Verificación rápida de estados y alarmas del cargador</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G97" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-03-S</t>
+        </is>
+      </c>
+      <c r="B98" s="7" t="inlineStr">
+        <is>
+          <t>CLG-03</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>Semanal</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores y chequeo visual de ventilación</t>
+        </is>
+      </c>
+      <c r="E98" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F98" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G98" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-03-M</t>
+        </is>
+      </c>
+      <c r="B99" s="7" t="inlineStr">
+        <is>
+          <t>CLG-03</t>
+        </is>
+      </c>
+      <c r="C99" s="7" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
+          <t>Limpieza de conectores, torque de bornes y prueba de carga completa</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G99" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-03-SE</t>
+        </is>
+      </c>
+      <c r="B100" s="7" t="inlineStr">
+        <is>
+          <t>CLG-03</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="inlineStr">
+        <is>
+          <t>Revisión termográfica de conexiones</t>
+        </is>
+      </c>
+      <c r="E100" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="F100" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G100" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="7" t="inlineStr">
+        <is>
+          <t>P-CLG-03-A</t>
+        </is>
+      </c>
+      <c r="B101" s="7" t="inlineStr">
+        <is>
+          <t>CLG-03</t>
+        </is>
+      </c>
+      <c r="C101" s="7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="D101" s="7" t="inlineStr">
+        <is>
+          <t>Mantención eléctrica mayor certificada</t>
+        </is>
+      </c>
+      <c r="E101" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="F101" s="7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/REEMPLAZAR/pautas-ELETTRIC80</t>
+        </is>
+      </c>
+      <c r="G101" s="7" t="inlineStr">
+        <is>
+          <t>Reemplazar el link por la pauta oficial del fabricante en Drive</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G1"/>
+  <dataValidations count="2">
+    <dataValidation sqref="B2:B5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>Maquinas!$A$2:$A$200</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>Listas!$H$2:$H$8</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>